<commit_message>
P2: record that a tick is evidence, and regenerate the workbook
D-256, and CLAUDE.md's four lines gain the two sentences that matter once a
year: the workbook is disposable, the database holds the record, and import
before re-exporting over a file because --force only ever loses ticks that
were never imported.

The committed workbook is regenerated in the new format - pre-filled tick
columns and a summary counted from the database rather than by a formula
Excel has to evaluate. Nothing was lost regenerating it: it held no ticks,
which is the last time that sentence will be true by luck rather than by
design.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/verification/Labourmax_verification.xlsx
+++ b/reference/verification/Labourmax_verification.xlsx
@@ -527,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>THIS WORKBOOK IS A WORK AID AND NEVER A SOURCE OF TRUTH. The fixtures in reference/ are the loaded data and docs/DECISIONS.md is the register; importverification records that a figure was checked and can never change one.</t>
+          <t>THIS WORKBOOK IS A WORK AID AND NEVER A SOURCE OF TRUTH. The fixtures in reference/ are the loaded data and docs/DECISIONS.md is the register; importverification records that a figure was checked and can never change one. The file itself is DISPOSABLE - every imported tick is in the database and is pre-filled on the next export. The counts below are as at export.</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,14 @@
       <c r="B6" t="n">
         <v>23</v>
       </c>
-      <c r="C6">
-        <f>COUNTIFS(Figures!$A:$A,$A6,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>COUNTIFS(Figures!$A:$A,$A6,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E6">
-        <f>$B6-$C6-$D6</f>
-        <v/>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -596,17 +593,14 @@
       <c r="B7" t="n">
         <v>67</v>
       </c>
-      <c r="C7">
-        <f>COUNTIFS(Figures!$A:$A,$A7,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>COUNTIFS(Figures!$A:$A,$A7,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E7">
-        <f>$B7-$C7-$D7</f>
-        <v/>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="8">
@@ -618,17 +612,14 @@
       <c r="B8" t="n">
         <v>86</v>
       </c>
-      <c r="C8">
-        <f>COUNTIFS(Figures!$A:$A,$A8,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D8">
-        <f>COUNTIFS(Figures!$A:$A,$A8,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E8">
-        <f>$B8-$C8-$D8</f>
-        <v/>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="9">
@@ -640,17 +631,14 @@
       <c r="B9" t="n">
         <v>2</v>
       </c>
-      <c r="C9">
-        <f>COUNTIFS(Figures!$A:$A,$A9,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>COUNTIFS(Figures!$A:$A,$A9,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E9">
-        <f>$B9-$C9-$D9</f>
-        <v/>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -662,17 +650,14 @@
       <c r="B10" t="n">
         <v>2</v>
       </c>
-      <c r="C10">
-        <f>COUNTIFS(Figures!$A:$A,$A10,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>COUNTIFS(Figures!$A:$A,$A10,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E10">
-        <f>$B10-$C10-$D10</f>
-        <v/>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -684,17 +669,14 @@
       <c r="B11" t="n">
         <v>2</v>
       </c>
-      <c r="C11">
-        <f>COUNTIFS(Figures!$A:$A,$A11,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D11">
-        <f>COUNTIFS(Figures!$A:$A,$A11,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E11">
-        <f>$B11-$C11-$D11</f>
-        <v/>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -706,17 +688,14 @@
       <c r="B12" t="n">
         <v>2</v>
       </c>
-      <c r="C12">
-        <f>COUNTIFS(Figures!$A:$A,$A12,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D12">
-        <f>COUNTIFS(Figures!$A:$A,$A12,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E12">
-        <f>$B12-$C12-$D12</f>
-        <v/>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -728,17 +707,14 @@
       <c r="B13" t="n">
         <v>8</v>
       </c>
-      <c r="C13">
-        <f>COUNTIFS(Figures!$A:$A,$A13,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D13">
-        <f>COUNTIFS(Figures!$A:$A,$A13,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>$B13-$C13-$D13</f>
-        <v/>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -750,17 +726,14 @@
       <c r="B14" t="n">
         <v>75</v>
       </c>
-      <c r="C14">
-        <f>COUNTIFS(Figures!$A:$A,$A14,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D14">
-        <f>COUNTIFS(Figures!$A:$A,$A14,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E14">
-        <f>$B14-$C14-$D14</f>
-        <v/>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="15">
@@ -772,17 +745,14 @@
       <c r="B15" t="n">
         <v>114</v>
       </c>
-      <c r="C15">
-        <f>COUNTIFS(Figures!$A:$A,$A15,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D15">
-        <f>COUNTIFS(Figures!$A:$A,$A15,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E15">
-        <f>$B15-$C15-$D15</f>
-        <v/>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>114</v>
       </c>
     </row>
     <row r="16">
@@ -794,17 +764,14 @@
       <c r="B16" t="n">
         <v>3</v>
       </c>
-      <c r="C16">
-        <f>COUNTIFS(Figures!$A:$A,$A16,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D16">
-        <f>COUNTIFS(Figures!$A:$A,$A16,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E16">
-        <f>$B16-$C16-$D16</f>
-        <v/>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -816,17 +783,14 @@
       <c r="B17" t="n">
         <v>12</v>
       </c>
-      <c r="C17">
-        <f>COUNTIFS(Figures!$A:$A,$A17,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D17">
-        <f>COUNTIFS(Figures!$A:$A,$A17,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E17">
-        <f>$B17-$C17-$D17</f>
-        <v/>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="18">
@@ -838,17 +802,14 @@
       <c r="B18" t="n">
         <v>36</v>
       </c>
-      <c r="C18">
-        <f>COUNTIFS(Figures!$A:$A,$A18,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D18">
-        <f>COUNTIFS(Figures!$A:$A,$A18,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E18">
-        <f>$B18-$C18-$D18</f>
-        <v/>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="19">
@@ -860,17 +821,14 @@
       <c r="B19" t="n">
         <v>67</v>
       </c>
-      <c r="C19">
-        <f>COUNTIFS(Figures!$A:$A,$A19,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D19">
-        <f>COUNTIFS(Figures!$A:$A,$A19,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E19">
-        <f>$B19-$C19-$D19</f>
-        <v/>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="20">
@@ -882,17 +840,14 @@
       <c r="B20" t="n">
         <v>66</v>
       </c>
-      <c r="C20">
-        <f>COUNTIFS(Figures!$A:$A,$A20,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>COUNTIFS(Figures!$A:$A,$A20,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>$B20-$C20-$D20</f>
-        <v/>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="21">
@@ -904,17 +859,14 @@
       <c r="B21" t="n">
         <v>4</v>
       </c>
-      <c r="C21">
-        <f>COUNTIFS(Figures!$A:$A,$A21,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D21">
-        <f>COUNTIFS(Figures!$A:$A,$A21,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E21">
-        <f>$B21-$C21-$D21</f>
-        <v/>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -926,17 +878,14 @@
       <c r="B22" t="n">
         <v>4</v>
       </c>
-      <c r="C22">
-        <f>COUNTIFS(Figures!$A:$A,$A22,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D22">
-        <f>COUNTIFS(Figures!$A:$A,$A22,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E22">
-        <f>$B22-$C22-$D22</f>
-        <v/>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -948,17 +897,14 @@
       <c r="B23" t="n">
         <v>2</v>
       </c>
-      <c r="C23">
-        <f>COUNTIFS(Figures!$A:$A,$A23,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D23">
-        <f>COUNTIFS(Figures!$A:$A,$A23,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E23">
-        <f>$B23-$C23-$D23</f>
-        <v/>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -970,17 +916,14 @@
       <c r="B24" t="n">
         <v>7</v>
       </c>
-      <c r="C24">
-        <f>COUNTIFS(Figures!$A:$A,$A24,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D24">
-        <f>COUNTIFS(Figures!$A:$A,$A24,Figures!$K:$K,"QUERY")</f>
-        <v/>
-      </c>
-      <c r="E24">
-        <f>$B24-$C24-$D24</f>
-        <v/>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -992,17 +935,14 @@
       <c r="B25" s="6" t="n">
         <v>582</v>
       </c>
-      <c r="C25" s="6">
-        <f>SUM(C6:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="6">
-        <f>SUM(D6:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="6">
-        <f>SUM(E6:E24)</f>
-        <v/>
+      <c r="C25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>582</v>
       </c>
     </row>
     <row r="27">
@@ -1058,13 +998,11 @@
       <c r="B29" t="n">
         <v>0</v>
       </c>
-      <c r="C29">
-        <f>COUNTIFS(Figures!$D:$D,$A29,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D29">
-        <f>COUNTIFS(Figures!$D:$D,$A29,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1091,13 +1029,11 @@
       <c r="B30" t="n">
         <v>114</v>
       </c>
-      <c r="C30">
-        <f>COUNTIFS(Figures!$D:$D,$A30,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D30">
-        <f>COUNTIFS(Figures!$D:$D,$A30,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1124,13 +1060,11 @@
       <c r="B31" t="n">
         <v>2</v>
       </c>
-      <c r="C31">
-        <f>COUNTIFS(Figures!$D:$D,$A31,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D31">
-        <f>COUNTIFS(Figures!$D:$D,$A31,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1157,13 +1091,11 @@
       <c r="B32" t="n">
         <v>2</v>
       </c>
-      <c r="C32">
-        <f>COUNTIFS(Figures!$D:$D,$A32,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D32">
-        <f>COUNTIFS(Figures!$D:$D,$A32,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1190,13 +1122,11 @@
       <c r="B33" t="n">
         <v>2</v>
       </c>
-      <c r="C33">
-        <f>COUNTIFS(Figures!$D:$D,$A33,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D33">
-        <f>COUNTIFS(Figures!$D:$D,$A33,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,13 +1153,11 @@
       <c r="B34" t="n">
         <v>12</v>
       </c>
-      <c r="C34">
-        <f>COUNTIFS(Figures!$D:$D,$A34,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D34">
-        <f>COUNTIFS(Figures!$D:$D,$A34,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1256,13 +1184,11 @@
       <c r="B35" t="n">
         <v>54</v>
       </c>
-      <c r="C35">
-        <f>COUNTIFS(Figures!$D:$D,$A35,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D35">
-        <f>COUNTIFS(Figures!$D:$D,$A35,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1289,13 +1215,11 @@
       <c r="B36" t="n">
         <v>7</v>
       </c>
-      <c r="C36">
-        <f>COUNTIFS(Figures!$D:$D,$A36,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D36">
-        <f>COUNTIFS(Figures!$D:$D,$A36,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1322,13 +1246,11 @@
       <c r="B37" t="n">
         <v>140</v>
       </c>
-      <c r="C37">
-        <f>COUNTIFS(Figures!$D:$D,$A37,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D37">
-        <f>COUNTIFS(Figures!$D:$D,$A37,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1355,13 +1277,11 @@
       <c r="B38" t="n">
         <v>2</v>
       </c>
-      <c r="C38">
-        <f>COUNTIFS(Figures!$D:$D,$A38,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D38">
-        <f>COUNTIFS(Figures!$D:$D,$A38,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1388,13 +1308,11 @@
       <c r="B39" t="n">
         <v>101</v>
       </c>
-      <c r="C39">
-        <f>COUNTIFS(Figures!$D:$D,$A39,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D39">
-        <f>COUNTIFS(Figures!$D:$D,$A39,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1421,13 +1339,11 @@
       <c r="B40" t="n">
         <v>52</v>
       </c>
-      <c r="C40">
-        <f>COUNTIFS(Figures!$D:$D,$A40,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D40">
-        <f>COUNTIFS(Figures!$D:$D,$A40,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1454,13 +1370,11 @@
       <c r="B41" t="n">
         <v>2</v>
       </c>
-      <c r="C41">
-        <f>COUNTIFS(Figures!$D:$D,$A41,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D41">
-        <f>COUNTIFS(Figures!$D:$D,$A41,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1487,13 +1401,11 @@
       <c r="B42" t="n">
         <v>2</v>
       </c>
-      <c r="C42">
-        <f>COUNTIFS(Figures!$D:$D,$A42,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D42">
-        <f>COUNTIFS(Figures!$D:$D,$A42,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1520,13 +1432,11 @@
       <c r="B43" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C43" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A43,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D43" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A43,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
@@ -1553,13 +1463,11 @@
       <c r="B44" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C44" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A44,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D44" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A44,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
@@ -1586,13 +1494,11 @@
       <c r="B45" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="C45" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A45,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D45" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A45,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
@@ -1619,13 +1525,11 @@
       <c r="B46" s="7" t="n">
         <v>56</v>
       </c>
-      <c r="C46" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A46,Figures!$K:$K,"Y")</f>
-        <v/>
-      </c>
-      <c r="D46" s="7">
-        <f>COUNTIFS(Figures!$D:$D,$A46,Figures!$K:$K,"QUERY")</f>
-        <v/>
+      <c r="C46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>

</xml_diff>